<commit_message>
Update listing data from workbook
</commit_message>
<xml_diff>
--- a/Office_Suites_NYC.xlsx
+++ b/Office_Suites_NYC.xlsx
@@ -8836,7 +8836,7 @@
       </c>
       <c r="O173" s="1" t="inlineStr">
         <is>
-          <t>833-410-3195</t>
+          <t>917-902-4421</t>
         </is>
       </c>
       <c r="Q173" s="2" t="inlineStr">
@@ -8899,7 +8899,7 @@
       </c>
       <c r="O174" s="1" t="inlineStr">
         <is>
-          <t>833-410-3195</t>
+          <t>917-902-4421</t>
         </is>
       </c>
       <c r="Q174" t="inlineStr">
@@ -8952,7 +8952,7 @@
       </c>
       <c r="O175" s="1" t="inlineStr">
         <is>
-          <t>833-410-3195</t>
+          <t>917-902-4421</t>
         </is>
       </c>
       <c r="AE175" t="inlineStr">
@@ -9000,7 +9000,7 @@
       </c>
       <c r="O176" s="1" t="inlineStr">
         <is>
-          <t>833-410-3195</t>
+          <t>917-902-4421</t>
         </is>
       </c>
       <c r="AE176" t="inlineStr">
@@ -9054,7 +9054,7 @@
       </c>
       <c r="O178" s="1" t="inlineStr">
         <is>
-          <t>646-320-89022</t>
+          <t>646-320-8922</t>
         </is>
       </c>
       <c r="Q178" s="2" t="inlineStr">
@@ -9123,12 +9123,17 @@
       </c>
       <c r="M180" s="8" t="inlineStr">
         <is>
-          <t>Yessenia</t>
+          <t>Paul Carter</t>
         </is>
       </c>
       <c r="O180" s="1" t="inlineStr">
         <is>
-          <t>917-574-9011</t>
+          <t>917-374-6111</t>
+        </is>
+      </c>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>pcarter@corporatesuites.com</t>
         </is>
       </c>
       <c r="U180" s="21" t="n">
@@ -9174,12 +9179,17 @@
       </c>
       <c r="M181" s="8" t="inlineStr">
         <is>
-          <t>Yessenia</t>
+          <t>Paul Carter</t>
         </is>
       </c>
       <c r="O181" s="1" t="inlineStr">
         <is>
-          <t>917-574-9011</t>
+          <t>917-374-6111</t>
+        </is>
+      </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>pcarter@corporatesuites.com</t>
         </is>
       </c>
       <c r="AE181" t="inlineStr">
@@ -9222,12 +9232,17 @@
       </c>
       <c r="M182" s="8" t="inlineStr">
         <is>
-          <t>Paul</t>
+          <t>Paul Carter</t>
         </is>
       </c>
       <c r="O182" s="1" t="inlineStr">
         <is>
-          <t>866-336-4581</t>
+          <t>917-374-6111</t>
+        </is>
+      </c>
+      <c r="Q182" t="inlineStr">
+        <is>
+          <t>pcarter@corporatesuites.com</t>
         </is>
       </c>
       <c r="AE182" t="inlineStr">
@@ -9270,12 +9285,17 @@
       </c>
       <c r="M183" s="8" t="inlineStr">
         <is>
-          <t>Yessenia</t>
+          <t>Paul Carter</t>
         </is>
       </c>
       <c r="O183" s="1" t="inlineStr">
         <is>
-          <t>917-574-9011</t>
+          <t>917-374-6111</t>
+        </is>
+      </c>
+      <c r="Q183" t="inlineStr">
+        <is>
+          <t>pcarter@corporatesuites.com</t>
         </is>
       </c>
       <c r="U183" t="inlineStr">
@@ -9294,10 +9314,19 @@
         <f>+A184+1</f>
         <v/>
       </c>
-      <c r="M184" s="8" t="n"/>
+      <c r="M184" s="8" t="inlineStr">
+        <is>
+          <t>Paul Carter</t>
+        </is>
+      </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t>tel:+18663364581</t>
+          <t>917-374-6111</t>
+        </is>
+      </c>
+      <c r="Q184" t="inlineStr">
+        <is>
+          <t>pcarter@corporatesuites.com</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Select Office Suites listings
</commit_message>
<xml_diff>
--- a/Office_Suites_NYC.xlsx
+++ b/Office_Suites_NYC.xlsx
@@ -696,7 +696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH311"/>
+  <dimension ref="A1:AH313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.140625" customWidth="1" min="1" max="2"/>
@@ -849,7 +849,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" t="n">
         <v>1</v>
@@ -12630,6 +12629,122 @@
       </c>
       <c r="AH311" s="28" t="n">
         <v>46296</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="n">
+        <v>221</v>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Select Office Suites</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>90 Broad Street, Floor 2, 3, 10</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>Financial District</t>
+        </is>
+      </c>
+      <c r="K312" t="n">
+        <v>10004</v>
+      </c>
+      <c r="M312" t="inlineStr">
+        <is>
+          <t>Rudy Maisto</t>
+        </is>
+      </c>
+      <c r="O312" t="inlineStr">
+        <is>
+          <t>646-461-9802</t>
+        </is>
+      </c>
+      <c r="Q312" t="inlineStr">
+        <is>
+          <t>rudy@selectofficesuites.com</t>
+        </is>
+      </c>
+      <c r="S312" t="inlineStr">
+        <is>
+          <t>www.selectofficesuites.com</t>
+        </is>
+      </c>
+      <c r="U312" t="inlineStr">
+        <is>
+          <t>Pays 10% commission first year, negotiable after</t>
+        </is>
+      </c>
+      <c r="AE312" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="n">
+        <v>222</v>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Select Office Suites</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>1115 Broadway (16 Madison Square West), Floor 9, 10, 11, 12</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>Manhattan</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>Flatiron District</t>
+        </is>
+      </c>
+      <c r="K313" t="n">
+        <v>10010</v>
+      </c>
+      <c r="M313" t="inlineStr">
+        <is>
+          <t>Rudy Maisto</t>
+        </is>
+      </c>
+      <c r="O313" t="inlineStr">
+        <is>
+          <t>646-461-9802</t>
+        </is>
+      </c>
+      <c r="Q313" t="inlineStr">
+        <is>
+          <t>rudy@selectofficesuites.com</t>
+        </is>
+      </c>
+      <c r="S313" t="inlineStr">
+        <is>
+          <t>www.selectofficesuites.com</t>
+        </is>
+      </c>
+      <c r="U313" t="inlineStr">
+        <is>
+          <t>Pays 10% commission first year, negotiable after</t>
+        </is>
+      </c>
+      <c r="AE313" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix duplicate 90 Broad Street listing
</commit_message>
<xml_diff>
--- a/Office_Suites_NYC.xlsx
+++ b/Office_Suites_NYC.xlsx
@@ -9334,110 +9334,32 @@
         <f>+A185+1</f>
         <v/>
       </c>
-      <c r="C185" s="1" t="inlineStr">
-        <is>
-          <t>Select Office Suites</t>
-        </is>
-      </c>
+      <c r="C185" s="1" t="n"/>
       <c r="D185" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E185" t="inlineStr">
-        <is>
-          <t>90 Boad Street, Floor 2, 3, 10</t>
-        </is>
-      </c>
-      <c r="G185" s="1" t="inlineStr">
-        <is>
-          <t>Manhattan</t>
-        </is>
-      </c>
-      <c r="I185" s="1" t="inlineStr">
-        <is>
-          <t>Financial District</t>
-        </is>
-      </c>
-      <c r="K185" s="1" t="n">
-        <v>10004</v>
-      </c>
-      <c r="M185" s="8" t="inlineStr">
-        <is>
-          <t>Rudy Maisto</t>
-        </is>
-      </c>
-      <c r="O185" s="1" t="inlineStr">
-        <is>
-          <t>646-461-9802</t>
-        </is>
-      </c>
-      <c r="Q185" s="2" t="inlineStr">
-        <is>
-          <t>rudy@selectofficesuites.com</t>
-        </is>
-      </c>
-      <c r="U185" t="inlineStr">
-        <is>
-          <t>first year 10% can work out longer term commission</t>
-        </is>
-      </c>
-      <c r="AE185" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="G185" s="1" t="n"/>
+      <c r="I185" s="1" t="n"/>
+      <c r="K185" s="1" t="n"/>
+      <c r="M185" s="8" t="n"/>
+      <c r="O185" s="1" t="n"/>
+      <c r="Q185" s="2" t="n"/>
     </row>
     <row r="186">
       <c r="A186">
         <f>+A186+1</f>
         <v/>
       </c>
-      <c r="C186" s="1" t="inlineStr">
-        <is>
-          <t>Select Office Suites</t>
-        </is>
-      </c>
+      <c r="C186" s="1" t="n"/>
       <c r="D186" s="1">
         <f>+D186+1</f>
         <v/>
       </c>
-      <c r="E186" t="inlineStr">
-        <is>
-          <t>1115 Braodway (15 Madison Ave West), Floor 9, 10, 11, 12</t>
-        </is>
-      </c>
-      <c r="G186" s="1" t="inlineStr">
-        <is>
-          <t>Manhattan</t>
-        </is>
-      </c>
-      <c r="I186" s="1" t="inlineStr">
-        <is>
-          <t>Flatiron / NoMad</t>
-        </is>
-      </c>
-      <c r="K186" s="1" t="n">
-        <v>10010</v>
-      </c>
-      <c r="M186" s="8" t="inlineStr">
-        <is>
-          <t>Rudy Maisto</t>
-        </is>
-      </c>
-      <c r="O186" s="1" t="inlineStr">
-        <is>
-          <t>646-461-9802</t>
-        </is>
-      </c>
-      <c r="Q186" t="inlineStr">
-        <is>
-          <t>mailto:rudy@selectofficesuites.com</t>
-        </is>
-      </c>
-      <c r="AE186" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="G186" s="1" t="n"/>
+      <c r="I186" s="1" t="n"/>
+      <c r="K186" s="1" t="n"/>
+      <c r="M186" s="8" t="n"/>
+      <c r="O186" s="1" t="n"/>
     </row>
     <row r="187">
       <c r="A187">
@@ -12823,8 +12745,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E183" display="https://www.corporatesuites.com/locations/880-third-avenue-shared-office-space-nyc/" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O183" display="tel:+18663364581" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O184" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q186" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U189" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U189" r:id="rId74"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix typos in listings
</commit_message>
<xml_diff>
--- a/Office_Suites_NYC.xlsx
+++ b/Office_Suites_NYC.xlsx
@@ -3188,7 +3188,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>159 West 25th street, floor 4, 5, 7, &amp; 8</t>
+          <t>159 West 25th Street, Floor 4, 5, 7, &amp; 8</t>
         </is>
       </c>
       <c r="G56" s="1" t="inlineStr">
@@ -4298,7 +4298,7 @@
       </c>
       <c r="U81" t="inlineStr">
         <is>
-          <t>he shows space and I don’t need to be present, 4th floor is currenly has spaces on iy</t>
+          <t>he shows space and I don’t need to be present, 4th floor currently has spaces on it</t>
         </is>
       </c>
       <c r="AE81" t="inlineStr">
@@ -4390,7 +4390,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>902 Braodway (June 2026 opening)</t>
+          <t>902 Broadway (June 2026 opening)</t>
         </is>
       </c>
       <c r="G84" s="1" t="inlineStr">
@@ -4655,7 +4655,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>390 park Avenue (June 2026 opening)</t>
+          <t>390 Park Avenue (June 2026 opening)</t>
         </is>
       </c>
       <c r="G89" s="1" t="inlineStr">
@@ -5369,7 +5369,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>215 Park Avnue South</t>
+          <t>215 Park Avenue South</t>
         </is>
       </c>
       <c r="G103" s="1" t="inlineStr">
@@ -5878,7 +5878,11 @@
       <c r="K113" s="1" t="n"/>
       <c r="M113" s="8" t="n"/>
       <c r="O113" s="1" t="n"/>
-      <c r="Q113" s="2" t="n"/>
+      <c r="Q113" s="2" t="inlineStr">
+        <is>
+          <t>mailto:brokers@industriousoffice.com</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -7240,7 +7244,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>575 Fith Avenue</t>
+          <t>575 Fifth Avenue</t>
         </is>
       </c>
       <c r="G143" s="1" t="inlineStr">
@@ -7938,7 +7942,7 @@
       </c>
       <c r="U159" t="inlineStr">
         <is>
-          <t>I don’t need to show space - cleitn can go direct</t>
+          <t>I don’t need to show space - client can go direct</t>
         </is>
       </c>
       <c r="AE159" t="inlineStr">
@@ -8744,8 +8748,10 @@
           <t>pcarter@corporatesuites.com</t>
         </is>
       </c>
-      <c r="U180" s="21" t="n">
-        <v>0.1</v>
+      <c r="U180" s="21" t="inlineStr">
+        <is>
+          <t>10% per year</t>
+        </is>
       </c>
       <c r="AE180" t="inlineStr">
         <is>
@@ -8902,7 +8908,7 @@
       </c>
       <c r="U183" t="inlineStr">
         <is>
-          <t>2 mos concious</t>
+          <t>2 months concession</t>
         </is>
       </c>
       <c r="AE183" t="inlineStr">

</xml_diff>

<commit_message>
Remove stale opening-date notes
</commit_message>
<xml_diff>
--- a/Office_Suites_NYC.xlsx
+++ b/Office_Suites_NYC.xlsx
@@ -4390,7 +4390,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>902 Broadway (June 2026 opening)</t>
+          <t>902 Broadway</t>
         </is>
       </c>
       <c r="G84" s="1" t="inlineStr">
@@ -4502,7 +4502,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>386 Park Avenue South  (June 2026 opening)</t>
+          <t>386 Park Avenue South</t>
         </is>
       </c>
       <c r="G86" s="1" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>875 Third Avenue (June 2026 opening)</t>
+          <t>875 Third Avenue</t>
         </is>
       </c>
       <c r="G88" s="1" t="inlineStr">
@@ -4655,7 +4655,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>390 Park Avenue (June 2026 opening)</t>
+          <t>390 Park Avenue</t>
         </is>
       </c>
       <c r="G89" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
       </c>
       <c r="E168" s="8" t="inlineStr">
         <is>
-          <t>717 Fifth Avenue, Floor 12A and 14 (opening in August 26)</t>
+          <t>717 Fifth Avenue, Floor 12A and 14</t>
         </is>
       </c>
       <c r="G168" s="1" t="inlineStr">
@@ -8875,7 +8875,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t xml:space="preserve">613 East 34th Street (opening up August 1), </t>
+          <t>613 East 34th Street</t>
         </is>
       </c>
       <c r="G183" s="1" t="inlineStr">

</xml_diff>